<commit_message>
Add in-app page help; reject thin source pages; replace an ungrounded item in the schedule
A How this page works panel under every page explains each section in plain language. The page reader now refuses pages with too little real article text (it had returned a site menu for one video page, so that item was removed and replaced). Workbook rebuilt to match the database.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/VeerNXT_Industry_Insights_Schedule.xlsx
+++ b/docs/VeerNXT_Industry_Insights_Schedule.xlsx
@@ -1818,21 +1818,21 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>Land Will Be the Currency of Victory in India • #GoodGenerals</t>
+          <t>Operation Dawn of Yemen and Saudi Arabia’s Available Options</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>Land plays a crucial role in India's strategic victories. Explore its significance in shaping counter-terror policies in the latest insights from CLAWS. How do you think land influences military strategy?</t>
+          <t>Operation Dawn in Yemen exposes the challenges of alliances. Saudi Arabia finds itself navigating regional complexities with limited international support. Check out CLAWS for detailed insights. #YemenConflict #MiddleEast</t>
         </is>
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>#IndiaDefence #VeteranInsights</t>
+          <t>#YemenConflict #MiddleEast</t>
         </is>
       </c>
       <c r="J17" s="15" t="n">
-        <v>204</v>
+        <v>221</v>
       </c>
       <c r="K17" s="15" t="inlineStr">
         <is>
@@ -1841,13 +1841,13 @@
       </c>
       <c r="L17" s="18" t="inlineStr">
         <is>
-          <t>https://claws.co.in/land-will-be-the-currency-of-victory-in-india-goodgenerals/</t>
+          <t>https://claws.co.in/operation-dawn-of-yemen-and-saudi-arabias-available-options/</t>
         </is>
       </c>
       <c r="M17" s="19" t="n"/>
       <c r="N17" s="19" t="n"/>
     </row>
-    <row r="18" ht="150" customHeight="1">
+    <row r="18" ht="165" customHeight="1">
       <c r="A18" s="15" t="n">
         <v>14</v>
       </c>
@@ -1872,22 +1872,21 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>Land Will Be the Currency of Victory in India • #GoodGenerals</t>
+          <t>Operation Dawn of Yemen and Saudi Arabia’s Available Options</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>In the intricate realm of national security, land remains a cornerstone of India's strategic victories. A recent article by CLAWS explores the geopolitical factors shaping our counter-terror policies. For Ex-Service Men (ESM), understanding these strategies can deepen their appreciation of the critical role land plays in national defense. How do you think these insights might influence the perspectives of veterans stepping into civilian roles?
-Explore the full article by CLAWS for more insights on this significant topic.</t>
+          <t>The recent developments in Yemen, particularly Operation Dawn, highlight the intricate and shifting alliances in the Middle East. As Saudi Arabia faces challenges with limited support from traditional allies, the importance of regional cooperation becomes evident. This scenario offers valuable insights for those interested in defence and security roles, emphasizing the need to understand geopolitical dynamics. How do you think these shifting alliances will impact regional stability in the long term? For more in-depth analysis, read the full article by CLAWS.</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>#IndiaDefence #VeteranInsights</t>
+          <t>#Geopolitics #MiddleEast #DefenceStrategy</t>
         </is>
       </c>
       <c r="J18" s="15" t="n">
-        <v>527</v>
+        <v>564</v>
       </c>
       <c r="K18" s="15" t="inlineStr">
         <is>
@@ -1896,13 +1895,13 @@
       </c>
       <c r="L18" s="18" t="inlineStr">
         <is>
-          <t>https://claws.co.in/land-will-be-the-currency-of-victory-in-india-goodgenerals/</t>
+          <t>https://claws.co.in/operation-dawn-of-yemen-and-saudi-arabias-available-options/</t>
         </is>
       </c>
       <c r="M18" s="19" t="n"/>
       <c r="N18" s="19" t="n"/>
     </row>
-    <row r="19" ht="75" customHeight="1">
+    <row r="19" ht="90" customHeight="1">
       <c r="A19" s="15" t="n">
         <v>15</v>
       </c>
@@ -1927,21 +1926,21 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>Land Will Be the Currency of Victory in India • #GoodGenerals</t>
+          <t>Operation Dawn of Yemen and Saudi Arabia’s Available Options</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>Did you know that land plays a crucial role in India's strategic defense? According to insights from CLAWS, it significantly impacts our counter-terror strategies. How do you think land should be managed to enhance national security?</t>
+          <t>Operation Dawn marks a crucial turning point in the Middle East as Saudi Arabia navigates complex alliances and strategic challenges. How do you think these developments will impact regional stability? For more insights, check out the detailed analysis by CLAWS.</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>#IndiaDefence #VeteranInsights #StrategicLeadership</t>
+          <t>#MiddleEast #DefenceStrategy #Geopolitics</t>
         </is>
       </c>
       <c r="J19" s="15" t="n">
-        <v>233</v>
+        <v>262</v>
       </c>
       <c r="K19" s="15" t="inlineStr">
         <is>
@@ -1950,7 +1949,7 @@
       </c>
       <c r="L19" s="18" t="inlineStr">
         <is>
-          <t>https://claws.co.in/land-will-be-the-currency-of-victory-in-india-goodgenerals/</t>
+          <t>https://claws.co.in/operation-dawn-of-yemen-and-saudi-arabias-available-options/</t>
         </is>
       </c>
       <c r="M19" s="19" t="n"/>
@@ -1981,22 +1980,21 @@
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>Land Will Be the Currency of Victory in India • #GoodGenerals</t>
+          <t>Operation Dawn of Yemen and Saudi Arabia’s Available Options</t>
         </is>
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>India's strategic victories are closely tied to the significance of land in our defense strategies. A thought-provoking article by CLAWS delves into how land impacts our counter-terror policies and geopolitical dynamics. For Ex-Service Men (ESM), these insights are crucial for understanding the broader picture of national security. What are your thoughts on the role of land in defense strategies? 
-Check out the full article for more details.</t>
+          <t>Operation Dawn of Yemen underscores the intricate alliances and evolving power dynamics in the Middle East. According to a report by CLAWS, Saudi Arabia's efforts to regain control from Ansar Allah reveal the challenges posed by limited support from traditional allies. This situation emphasizes the importance of strategic regional partnerships. How do you think these geopolitical changes might affect global security? Share your thoughts with us!</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>#IndiaDefence #VeteranInsights</t>
+          <t>#Geopolitics #YemenConflict</t>
         </is>
       </c>
       <c r="J20" s="15" t="n">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="K20" s="15" t="inlineStr">
         <is>
@@ -2005,7 +2003,7 @@
       </c>
       <c r="L20" s="18" t="inlineStr">
         <is>
-          <t>https://claws.co.in/land-will-be-the-currency-of-victory-in-india-goodgenerals/</t>
+          <t>https://claws.co.in/operation-dawn-of-yemen-and-saudi-arabias-available-options/</t>
         </is>
       </c>
       <c r="M20" s="19" t="n"/>
@@ -3762,7 +3760,7 @@
       <c r="B8" s="10" t="n"/>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Land Will Be the Currency of Victory in India • #GoodGenerals</t>
+          <t>Operation Dawn of Yemen and Saudi Arabia’s Available Options</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -3772,18 +3770,18 @@
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Centre for Land Warfare Studies (CLAWS)</t>
+          <t>Suyash Dwivedi</t>
         </is>
       </c>
       <c r="F8" s="20" t="n">
-        <v>46296.16770833333</v>
+        <v>46308.60071759259</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>https://claws.co.in/land-will-be-the-currency-of-victory-in-india-goodgenerals/</t>
+          <t>https://claws.co.in/operation-dawn-of-yemen-and-saudi-arabias-available-options/</t>
         </is>
       </c>
       <c r="I8" s="10" t="n">
@@ -4092,10 +4090,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="49" customHeight="1">
+    <row r="7" ht="79" customHeight="1">
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>One article was deliberately dropped: "The Forgotten Rights of those in Uniform" (IMR Media). It concerns police conduct during political protests and does not mention Ex-Service Men, so it is not suitable for us to comment on.</t>
+          <t>Two articles were deliberately dropped. "The Forgotten Rights of those in Uniform" (IMR Media) concerns police conduct during political protests and does not mention Ex-Service Men, so it is not suitable for us to comment on. "Land Will Be the Currency of Victory in India" (CLAWS) is mostly a video page with almost no article text, so posts could not be grounded in it; it was replaced by "Operation Dawn of Yemen and Saudi Arabia's Available Options" (CLAWS).</t>
         </is>
       </c>
     </row>
@@ -4107,10 +4105,10 @@
       </c>
       <c r="B8" s="22" t="n"/>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Each post was written from the full text of the article, in new wording, with the source credited.</t>
+          <t>Each post was written from the full text of the article, in new wording, with the source credited. The tool now refuses pages that contain too little real article text.</t>
         </is>
       </c>
     </row>
@@ -4153,7 +4151,7 @@
     <row r="15" ht="34" customHeight="1">
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Topics: most articles are about strategy and technology, not directly about veterans. The two closest to our audience are the 8th Pay Commission and the dual-use technology pieces.</t>
+          <t>Topics: most articles are about strategy and technology, not directly about veterans. The one closest to our audience is the 8th Pay Commission piece.</t>
         </is>
       </c>
     </row>

</xml_diff>